<commit_message>
Dashboard: 2026-09-23 14:34 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1063,11 +1063,11 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -2267,11 +2267,11 @@
         <v>9</v>
       </c>
       <c r="E100" t="n">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4675,11 @@
         <v>9</v>
       </c>
       <c r="E232" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -5277,11 +5277,11 @@
         <v>9</v>
       </c>
       <c r="E265" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -5879,11 +5879,11 @@
         <v>9</v>
       </c>
       <c r="E298" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -5893,11 +5893,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B299" t="inlineStr"/>
       <c r="C299" t="n">
         <v>2024</v>
       </c>
@@ -5907,11 +5903,7 @@
       <c r="E299" t="n">
         <v>354</v>
       </c>
-      <c r="F299" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -5919,11 +5911,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B300" t="inlineStr"/>
       <c r="C300" t="n">
         <v>2024</v>
       </c>
@@ -5933,11 +5921,7 @@
       <c r="E300" t="n">
         <v>154</v>
       </c>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -5945,11 +5929,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B301" t="inlineStr"/>
       <c r="C301" t="n">
         <v>2024</v>
       </c>
@@ -5959,11 +5939,7 @@
       <c r="E301" t="n">
         <v>158</v>
       </c>
-      <c r="F301" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -5971,11 +5947,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B302" t="inlineStr"/>
       <c r="C302" t="n">
         <v>2024</v>
       </c>
@@ -5985,11 +5957,7 @@
       <c r="E302" t="n">
         <v>356</v>
       </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -5997,11 +5965,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B303" t="inlineStr"/>
       <c r="C303" t="n">
         <v>2024</v>
       </c>
@@ -6011,11 +5975,7 @@
       <c r="E303" t="n">
         <v>553</v>
       </c>
-      <c r="F303" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -6023,11 +5983,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B304" t="inlineStr"/>
       <c r="C304" t="n">
         <v>2024</v>
       </c>
@@ -6037,11 +5993,7 @@
       <c r="E304" t="n">
         <v>399</v>
       </c>
-      <c r="F304" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -6049,11 +6001,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B305" t="inlineStr"/>
       <c r="C305" t="n">
         <v>2024</v>
       </c>
@@ -6063,11 +6011,7 @@
       <c r="E305" t="n">
         <v>132</v>
       </c>
-      <c r="F305" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -6075,11 +6019,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B306" t="inlineStr"/>
       <c r="C306" t="n">
         <v>2024</v>
       </c>
@@ -6089,11 +6029,7 @@
       <c r="E306" t="n">
         <v>349</v>
       </c>
-      <c r="F306" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -6101,11 +6037,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B307" t="inlineStr"/>
       <c r="C307" t="n">
         <v>2024</v>
       </c>
@@ -6115,11 +6047,7 @@
       <c r="E307" t="n">
         <v>353</v>
       </c>
-      <c r="F307" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -6127,11 +6055,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B308" t="inlineStr"/>
       <c r="C308" t="n">
         <v>2024</v>
       </c>
@@ -6141,11 +6065,7 @@
       <c r="E308" t="n">
         <v>288</v>
       </c>
-      <c r="F308" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -6153,11 +6073,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B309" t="inlineStr"/>
       <c r="C309" t="n">
         <v>2024</v>
       </c>
@@ -6167,11 +6083,7 @@
       <c r="E309" t="n">
         <v>235</v>
       </c>
-      <c r="F309" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -6179,11 +6091,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B310" t="inlineStr"/>
       <c r="C310" t="n">
         <v>2024</v>
       </c>
@@ -6193,11 +6101,7 @@
       <c r="E310" t="n">
         <v>390</v>
       </c>
-      <c r="F310" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -6205,11 +6109,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B311" t="inlineStr"/>
       <c r="C311" t="n">
         <v>2025</v>
       </c>
@@ -6219,11 +6119,7 @@
       <c r="E311" t="n">
         <v>565</v>
       </c>
-      <c r="F311" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -6231,11 +6127,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B312" t="inlineStr"/>
       <c r="C312" t="n">
         <v>2025</v>
       </c>
@@ -6245,11 +6137,7 @@
       <c r="E312" t="n">
         <v>425</v>
       </c>
-      <c r="F312" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -6257,11 +6145,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B313" t="inlineStr"/>
       <c r="C313" t="n">
         <v>2025</v>
       </c>
@@ -6271,11 +6155,7 @@
       <c r="E313" t="n">
         <v>396</v>
       </c>
-      <c r="F313" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -6283,11 +6163,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B314" t="inlineStr"/>
       <c r="C314" t="n">
         <v>2025</v>
       </c>
@@ -6297,11 +6173,7 @@
       <c r="E314" t="n">
         <v>327</v>
       </c>
-      <c r="F314" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -6309,11 +6181,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B315" t="inlineStr"/>
       <c r="C315" t="n">
         <v>2025</v>
       </c>
@@ -6323,11 +6191,7 @@
       <c r="E315" t="n">
         <v>367</v>
       </c>
-      <c r="F315" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -6335,11 +6199,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B316" t="inlineStr"/>
       <c r="C316" t="n">
         <v>2025</v>
       </c>
@@ -6349,11 +6209,7 @@
       <c r="E316" t="n">
         <v>281</v>
       </c>
-      <c r="F316" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -6361,11 +6217,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B317" t="inlineStr"/>
       <c r="C317" t="n">
         <v>2025</v>
       </c>
@@ -6375,11 +6227,7 @@
       <c r="E317" t="n">
         <v>321</v>
       </c>
-      <c r="F317" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -6387,11 +6235,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B318" t="inlineStr"/>
       <c r="C318" t="n">
         <v>2025</v>
       </c>
@@ -6401,11 +6245,7 @@
       <c r="E318" t="n">
         <v>301</v>
       </c>
-      <c r="F318" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -6413,11 +6253,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B319" t="inlineStr"/>
       <c r="C319" t="n">
         <v>2025</v>
       </c>
@@ -6427,11 +6263,7 @@
       <c r="E319" t="n">
         <v>420</v>
       </c>
-      <c r="F319" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -6439,11 +6271,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B320" t="inlineStr"/>
       <c r="C320" t="n">
         <v>2025</v>
       </c>
@@ -6453,11 +6281,7 @@
       <c r="E320" t="n">
         <v>355</v>
       </c>
-      <c r="F320" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -6465,11 +6289,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B321" t="inlineStr"/>
       <c r="C321" t="n">
         <v>2025</v>
       </c>
@@ -6479,11 +6299,7 @@
       <c r="E321" t="n">
         <v>311</v>
       </c>
-      <c r="F321" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -6491,11 +6307,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B322" t="inlineStr"/>
       <c r="C322" t="n">
         <v>2025</v>
       </c>
@@ -6505,11 +6317,7 @@
       <c r="E322" t="n">
         <v>167</v>
       </c>
-      <c r="F322" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -6517,11 +6325,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B323" t="inlineStr"/>
       <c r="C323" t="n">
         <v>2026</v>
       </c>
@@ -6531,11 +6335,7 @@
       <c r="E323" t="n">
         <v>346</v>
       </c>
-      <c r="F323" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -6543,11 +6343,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B324" t="inlineStr"/>
       <c r="C324" t="n">
         <v>2026</v>
       </c>
@@ -6557,11 +6353,7 @@
       <c r="E324" t="n">
         <v>215</v>
       </c>
-      <c r="F324" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -6569,11 +6361,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B325" t="inlineStr"/>
       <c r="C325" t="n">
         <v>2026</v>
       </c>
@@ -6583,11 +6371,7 @@
       <c r="E325" t="n">
         <v>236</v>
       </c>
-      <c r="F325" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -6595,11 +6379,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B326" t="inlineStr"/>
       <c r="C326" t="n">
         <v>2026</v>
       </c>
@@ -6609,11 +6389,7 @@
       <c r="E326" t="n">
         <v>222</v>
       </c>
-      <c r="F326" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -6621,11 +6397,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B327" t="inlineStr"/>
       <c r="C327" t="n">
         <v>2026</v>
       </c>
@@ -6635,11 +6407,7 @@
       <c r="E327" t="n">
         <v>215</v>
       </c>
-      <c r="F327" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -6647,11 +6415,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B328" t="inlineStr"/>
       <c r="C328" t="n">
         <v>2026</v>
       </c>
@@ -6661,11 +6425,7 @@
       <c r="E328" t="n">
         <v>212</v>
       </c>
-      <c r="F328" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -6673,11 +6433,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B329" t="inlineStr"/>
       <c r="C329" t="n">
         <v>2026</v>
       </c>
@@ -6687,11 +6443,7 @@
       <c r="E329" t="n">
         <v>247</v>
       </c>
-      <c r="F329" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -6699,11 +6451,7 @@
           <t>Joquei</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B330" t="inlineStr"/>
       <c r="C330" t="n">
         <v>2026</v>
       </c>
@@ -6713,11 +6461,7 @@
       <c r="E330" t="n">
         <v>250</v>
       </c>
-      <c r="F330" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -6737,11 +6481,11 @@
         <v>9</v>
       </c>
       <c r="E331" t="n">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -6751,11 +6495,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B332" t="inlineStr"/>
       <c r="C332" t="n">
         <v>2024</v>
       </c>
@@ -6765,11 +6505,7 @@
       <c r="E332" t="n">
         <v>111</v>
       </c>
-      <c r="F332" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -6777,11 +6513,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B333" t="inlineStr"/>
       <c r="C333" t="n">
         <v>2024</v>
       </c>
@@ -6791,11 +6523,7 @@
       <c r="E333" t="n">
         <v>217</v>
       </c>
-      <c r="F333" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -6803,11 +6531,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B334" t="inlineStr"/>
       <c r="C334" t="n">
         <v>2024</v>
       </c>
@@ -6817,11 +6541,7 @@
       <c r="E334" t="n">
         <v>173</v>
       </c>
-      <c r="F334" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -6829,11 +6549,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B335" t="inlineStr"/>
       <c r="C335" t="n">
         <v>2024</v>
       </c>
@@ -6843,11 +6559,7 @@
       <c r="E335" t="n">
         <v>157</v>
       </c>
-      <c r="F335" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -6855,11 +6567,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B336" t="inlineStr"/>
       <c r="C336" t="n">
         <v>2024</v>
       </c>
@@ -6869,11 +6577,7 @@
       <c r="E336" t="n">
         <v>178</v>
       </c>
-      <c r="F336" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -6881,11 +6585,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B337" t="inlineStr"/>
       <c r="C337" t="n">
         <v>2024</v>
       </c>
@@ -6895,11 +6595,7 @@
       <c r="E337" t="n">
         <v>181</v>
       </c>
-      <c r="F337" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -6907,11 +6603,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B338" t="inlineStr"/>
       <c r="C338" t="n">
         <v>2024</v>
       </c>
@@ -6921,11 +6613,7 @@
       <c r="E338" t="n">
         <v>169</v>
       </c>
-      <c r="F338" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -6933,11 +6621,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B339" t="inlineStr"/>
       <c r="C339" t="n">
         <v>2024</v>
       </c>
@@ -6947,11 +6631,7 @@
       <c r="E339" t="n">
         <v>183</v>
       </c>
-      <c r="F339" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -6959,11 +6639,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B340" t="inlineStr"/>
       <c r="C340" t="n">
         <v>2024</v>
       </c>
@@ -6973,11 +6649,7 @@
       <c r="E340" t="n">
         <v>212</v>
       </c>
-      <c r="F340" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -6985,11 +6657,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B341" t="inlineStr"/>
       <c r="C341" t="n">
         <v>2024</v>
       </c>
@@ -6999,11 +6667,7 @@
       <c r="E341" t="n">
         <v>177</v>
       </c>
-      <c r="F341" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -7011,11 +6675,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B342" t="inlineStr"/>
       <c r="C342" t="n">
         <v>2024</v>
       </c>
@@ -7025,11 +6685,7 @@
       <c r="E342" t="n">
         <v>141</v>
       </c>
-      <c r="F342" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -7037,11 +6693,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B343" t="inlineStr"/>
       <c r="C343" t="n">
         <v>2024</v>
       </c>
@@ -7051,11 +6703,7 @@
       <c r="E343" t="n">
         <v>181</v>
       </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -7063,11 +6711,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B344" t="inlineStr"/>
       <c r="C344" t="n">
         <v>2025</v>
       </c>
@@ -7077,11 +6721,7 @@
       <c r="E344" t="n">
         <v>362</v>
       </c>
-      <c r="F344" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -7089,11 +6729,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B345" t="inlineStr"/>
       <c r="C345" t="n">
         <v>2025</v>
       </c>
@@ -7103,11 +6739,7 @@
       <c r="E345" t="n">
         <v>233</v>
       </c>
-      <c r="F345" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -7115,11 +6747,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B346" t="inlineStr"/>
       <c r="C346" t="n">
         <v>2025</v>
       </c>
@@ -7129,11 +6757,7 @@
       <c r="E346" t="n">
         <v>290</v>
       </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -7141,11 +6765,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B347" t="inlineStr"/>
       <c r="C347" t="n">
         <v>2025</v>
       </c>
@@ -7155,11 +6775,7 @@
       <c r="E347" t="n">
         <v>339</v>
       </c>
-      <c r="F347" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -7167,11 +6783,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B348" t="inlineStr"/>
       <c r="C348" t="n">
         <v>2025</v>
       </c>
@@ -7181,11 +6793,7 @@
       <c r="E348" t="n">
         <v>337</v>
       </c>
-      <c r="F348" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -7193,11 +6801,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B349" t="inlineStr"/>
       <c r="C349" t="n">
         <v>2025</v>
       </c>
@@ -7207,11 +6811,7 @@
       <c r="E349" t="n">
         <v>304</v>
       </c>
-      <c r="F349" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -7219,11 +6819,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B350" t="inlineStr"/>
       <c r="C350" t="n">
         <v>2025</v>
       </c>
@@ -7233,11 +6829,7 @@
       <c r="E350" t="n">
         <v>309</v>
       </c>
-      <c r="F350" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -7245,11 +6837,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B351" t="inlineStr"/>
       <c r="C351" t="n">
         <v>2025</v>
       </c>
@@ -7259,11 +6847,7 @@
       <c r="E351" t="n">
         <v>331</v>
       </c>
-      <c r="F351" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -7271,11 +6855,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B352" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B352" t="inlineStr"/>
       <c r="C352" t="n">
         <v>2025</v>
       </c>
@@ -7285,11 +6865,7 @@
       <c r="E352" t="n">
         <v>328</v>
       </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -7297,11 +6873,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B353" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B353" t="inlineStr"/>
       <c r="C353" t="n">
         <v>2025</v>
       </c>
@@ -7311,11 +6883,7 @@
       <c r="E353" t="n">
         <v>326</v>
       </c>
-      <c r="F353" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -7323,11 +6891,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B354" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B354" t="inlineStr"/>
       <c r="C354" t="n">
         <v>2025</v>
       </c>
@@ -7337,11 +6901,7 @@
       <c r="E354" t="n">
         <v>298</v>
       </c>
-      <c r="F354" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -7349,11 +6909,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B355" t="inlineStr"/>
       <c r="C355" t="n">
         <v>2025</v>
       </c>
@@ -7363,11 +6919,7 @@
       <c r="E355" t="n">
         <v>227</v>
       </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -7375,11 +6927,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B356" t="inlineStr"/>
       <c r="C356" t="n">
         <v>2026</v>
       </c>
@@ -7389,11 +6937,7 @@
       <c r="E356" t="n">
         <v>363</v>
       </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -7401,11 +6945,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B357" t="inlineStr"/>
       <c r="C357" t="n">
         <v>2026</v>
       </c>
@@ -7415,11 +6955,7 @@
       <c r="E357" t="n">
         <v>252</v>
       </c>
-      <c r="F357" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -7427,11 +6963,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B358" t="inlineStr"/>
       <c r="C358" t="n">
         <v>2026</v>
       </c>
@@ -7441,11 +6973,7 @@
       <c r="E358" t="n">
         <v>289</v>
       </c>
-      <c r="F358" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -7453,11 +6981,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B359" t="inlineStr"/>
       <c r="C359" t="n">
         <v>2026</v>
       </c>
@@ -7467,11 +6991,7 @@
       <c r="E359" t="n">
         <v>272</v>
       </c>
-      <c r="F359" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -7479,11 +6999,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B360" t="inlineStr"/>
       <c r="C360" t="n">
         <v>2026</v>
       </c>
@@ -7493,11 +7009,7 @@
       <c r="E360" t="n">
         <v>255</v>
       </c>
-      <c r="F360" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -7505,11 +7017,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B361" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B361" t="inlineStr"/>
       <c r="C361" t="n">
         <v>2026</v>
       </c>
@@ -7519,11 +7027,7 @@
       <c r="E361" t="n">
         <v>198</v>
       </c>
-      <c r="F361" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -7531,11 +7035,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B362" t="inlineStr"/>
       <c r="C362" t="n">
         <v>2026</v>
       </c>
@@ -7545,11 +7045,7 @@
       <c r="E362" t="n">
         <v>278</v>
       </c>
-      <c r="F362" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -7557,11 +7053,7 @@
           <t>Kennedy</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr">
-        <is>
-          <t>Regiao 2</t>
-        </is>
-      </c>
+      <c r="B363" t="inlineStr"/>
       <c r="C363" t="n">
         <v>2026</v>
       </c>
@@ -7571,11 +7063,7 @@
       <c r="E363" t="n">
         <v>278</v>
       </c>
-      <c r="F363" t="inlineStr">
-        <is>
-          <t>2026-09-22 11:17</t>
-        </is>
-      </c>
+      <c r="F363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -7595,11 +7083,11 @@
         <v>9</v>
       </c>
       <c r="E364" t="n">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -8197,11 +7685,11 @@
         <v>9</v>
       </c>
       <c r="E397" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -8799,11 +8287,11 @@
         <v>9</v>
       </c>
       <c r="E430" t="n">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -9401,11 +8889,11 @@
         <v>9</v>
       </c>
       <c r="E463" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -10003,11 +9491,11 @@
         <v>9</v>
       </c>
       <c r="E496" t="n">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -10605,11 +10093,11 @@
         <v>9</v>
       </c>
       <c r="E529" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -11207,11 +10695,11 @@
         <v>9</v>
       </c>
       <c r="E562" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -11809,11 +11297,11 @@
         <v>9</v>
       </c>
       <c r="E595" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -12415,7 +11903,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -13013,11 +12501,11 @@
         <v>9</v>
       </c>
       <c r="E661" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -13615,11 +13103,11 @@
         <v>9</v>
       </c>
       <c r="E694" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -14217,11 +13705,11 @@
         <v>9</v>
       </c>
       <c r="E727" t="n">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -14819,11 +14307,11 @@
         <v>9</v>
       </c>
       <c r="E760" t="n">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -15425,7 +14913,7 @@
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>2026-09-22 11:17</t>
+          <t>2026-09-23 11:33</t>
         </is>
       </c>
     </row>
@@ -15754,7 +15242,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>694</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3">
@@ -15764,103 +15252,103 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>371</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>331</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>513</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>731</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>580</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>301</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>532</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>565</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>376</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>571</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>927</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>658</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>686</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>666</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>704</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>585</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>630</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>632</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>748</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>681</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>609</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>394</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>709</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>467</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
-        <v>525</v>
+        <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>494</v>
+        <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="AE3" t="n">
-        <v>410</v>
+        <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>525</v>
+        <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>528</v>
+        <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>798</v>
+        <v>851</v>
       </c>
     </row>
     <row r="4">
@@ -15966,7 +15454,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>570</v>
+        <v>599</v>
       </c>
     </row>
     <row r="5">
@@ -16072,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>678</v>
+        <v>691</v>
       </c>
     </row>
     <row r="6">
@@ -16178,7 +15666,7 @@
         <v>4248</v>
       </c>
       <c r="AH6" t="n">
-        <v>2740</v>
+        <v>2861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-09-24 14:32 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1063,11 +1063,11 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -2267,11 +2267,11 @@
         <v>9</v>
       </c>
       <c r="E100" t="n">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4073,11 @@
         <v>9</v>
       </c>
       <c r="E199" t="n">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4675,11 @@
         <v>9</v>
       </c>
       <c r="E232" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -5277,11 +5277,11 @@
         <v>9</v>
       </c>
       <c r="E265" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -6481,11 +6481,11 @@
         <v>9</v>
       </c>
       <c r="E331" t="n">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -7083,11 +7083,11 @@
         <v>9</v>
       </c>
       <c r="E364" t="n">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -7685,11 +7685,11 @@
         <v>9</v>
       </c>
       <c r="E397" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -8287,11 +8287,11 @@
         <v>9</v>
       </c>
       <c r="E430" t="n">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -8889,11 +8889,11 @@
         <v>9</v>
       </c>
       <c r="E463" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -9491,11 +9491,11 @@
         <v>9</v>
       </c>
       <c r="E496" t="n">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -10093,11 +10093,11 @@
         <v>9</v>
       </c>
       <c r="E529" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -10695,11 +10695,11 @@
         <v>9</v>
       </c>
       <c r="E562" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -11297,11 +11297,11 @@
         <v>9</v>
       </c>
       <c r="E595" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -11899,11 +11899,11 @@
         <v>9</v>
       </c>
       <c r="E628" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -12501,11 +12501,11 @@
         <v>9</v>
       </c>
       <c r="E661" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -13103,11 +13103,11 @@
         <v>9</v>
       </c>
       <c r="E694" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -13705,11 +13705,11 @@
         <v>9</v>
       </c>
       <c r="E727" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -14307,11 +14307,11 @@
         <v>9</v>
       </c>
       <c r="E760" t="n">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -14909,11 +14909,11 @@
         <v>9</v>
       </c>
       <c r="E793" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>2026-09-23 11:33</t>
+          <t>2026-09-24 11:30</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>720</v>
+        <v>750</v>
       </c>
     </row>
     <row r="3">
@@ -15348,7 +15348,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>851</v>
+        <v>890</v>
       </c>
     </row>
     <row r="4">
@@ -15454,7 +15454,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>599</v>
+        <v>630</v>
       </c>
     </row>
     <row r="5">
@@ -15560,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>691</v>
+        <v>710</v>
       </c>
     </row>
     <row r="6">
@@ -15666,7 +15666,7 @@
         <v>4248</v>
       </c>
       <c r="AH6" t="n">
-        <v>2861</v>
+        <v>2980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-09-25 14:54 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1063,11 +1063,11 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
-        <v>364</v>
+        <v>382</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -2267,11 +2267,11 @@
         <v>9</v>
       </c>
       <c r="E100" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4073,11 @@
         <v>9</v>
       </c>
       <c r="E199" t="n">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4675,11 @@
         <v>9</v>
       </c>
       <c r="E232" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -5277,11 +5277,11 @@
         <v>9</v>
       </c>
       <c r="E265" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -5879,11 +5879,11 @@
         <v>9</v>
       </c>
       <c r="E298" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -6481,11 +6481,11 @@
         <v>9</v>
       </c>
       <c r="E331" t="n">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -7083,11 +7083,11 @@
         <v>9</v>
       </c>
       <c r="E364" t="n">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -7685,11 +7685,11 @@
         <v>9</v>
       </c>
       <c r="E397" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -8287,11 +8287,11 @@
         <v>9</v>
       </c>
       <c r="E430" t="n">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -8889,11 +8889,11 @@
         <v>9</v>
       </c>
       <c r="E463" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -9491,11 +9491,11 @@
         <v>9</v>
       </c>
       <c r="E496" t="n">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -10093,11 +10093,11 @@
         <v>9</v>
       </c>
       <c r="E529" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -10695,11 +10695,11 @@
         <v>9</v>
       </c>
       <c r="E562" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -11297,11 +11297,11 @@
         <v>9</v>
       </c>
       <c r="E595" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -11899,11 +11899,11 @@
         <v>9</v>
       </c>
       <c r="E628" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -12501,11 +12501,11 @@
         <v>9</v>
       </c>
       <c r="E661" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -13103,11 +13103,11 @@
         <v>9</v>
       </c>
       <c r="E694" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -13705,11 +13705,11 @@
         <v>9</v>
       </c>
       <c r="E727" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -14307,11 +14307,11 @@
         <v>9</v>
       </c>
       <c r="E760" t="n">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -14913,7 +14913,7 @@
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>2026-09-24 11:30</t>
+          <t>2026-09-25 11:53</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>750</v>
+        <v>772</v>
       </c>
     </row>
     <row r="3">
@@ -15348,7 +15348,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>890</v>
+        <v>929</v>
       </c>
     </row>
     <row r="4">
@@ -15454,7 +15454,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>630</v>
+        <v>652</v>
       </c>
     </row>
     <row r="5">
@@ -15560,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>710</v>
+        <v>735</v>
       </c>
     </row>
     <row r="6">
@@ -15666,7 +15666,7 @@
         <v>4248</v>
       </c>
       <c r="AH6" t="n">
-        <v>2980</v>
+        <v>3088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-10-08 17:08 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1081,11 +1081,11 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -1701,11 +1701,11 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -2321,11 +2321,11 @@
         <v>10</v>
       </c>
       <c r="E103" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -3561,11 +3561,11 @@
         <v>10</v>
       </c>
       <c r="E171" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -4181,11 +4181,11 @@
         <v>10</v>
       </c>
       <c r="E205" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -4801,11 +4801,11 @@
         <v>10</v>
       </c>
       <c r="E239" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -5421,11 +5421,11 @@
         <v>10</v>
       </c>
       <c r="E273" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -6041,11 +6041,11 @@
         <v>10</v>
       </c>
       <c r="E307" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -6661,11 +6661,11 @@
         <v>10</v>
       </c>
       <c r="E341" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -7281,11 +7281,11 @@
         <v>10</v>
       </c>
       <c r="E375" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -7901,11 +7901,11 @@
         <v>10</v>
       </c>
       <c r="E409" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -8521,11 +8521,11 @@
         <v>10</v>
       </c>
       <c r="E443" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -9141,11 +9141,11 @@
         <v>10</v>
       </c>
       <c r="E477" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -9761,11 +9761,11 @@
         <v>10</v>
       </c>
       <c r="E511" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -10381,11 +10381,11 @@
         <v>10</v>
       </c>
       <c r="E545" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -11001,11 +11001,11 @@
         <v>10</v>
       </c>
       <c r="E579" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F579" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -11621,11 +11621,11 @@
         <v>10</v>
       </c>
       <c r="E613" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -12241,11 +12241,11 @@
         <v>10</v>
       </c>
       <c r="E647" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -12861,11 +12861,11 @@
         <v>10</v>
       </c>
       <c r="E681" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F681" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -13481,11 +13481,11 @@
         <v>10</v>
       </c>
       <c r="E715" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -14101,11 +14101,11 @@
         <v>10</v>
       </c>
       <c r="E749" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -14721,11 +14721,11 @@
         <v>10</v>
       </c>
       <c r="E783" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -15341,11 +15341,11 @@
         <v>10</v>
       </c>
       <c r="E817" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F817" t="inlineStr">
         <is>
-          <t>2026-10-07 14:07</t>
+          <t>2026-10-08 14:06</t>
         </is>
       </c>
     </row>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>167</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3">
@@ -15792,7 +15792,7 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>195</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
@@ -15901,7 +15901,7 @@
         <v>0</v>
       </c>
       <c r="AI4" t="n">
-        <v>114</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
@@ -16010,7 +16010,7 @@
         <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>130</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6">
@@ -16119,7 +16119,7 @@
         <v>3555</v>
       </c>
       <c r="AI6" t="n">
-        <v>606</v>
+        <v>733</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-10-20 14:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1081,11 +1081,11 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -1701,11 +1701,11 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -2321,11 +2321,11 @@
         <v>10</v>
       </c>
       <c r="E103" t="n">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -3561,11 +3561,11 @@
         <v>10</v>
       </c>
       <c r="E171" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -4181,11 +4181,11 @@
         <v>10</v>
       </c>
       <c r="E205" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -4801,11 +4801,11 @@
         <v>10</v>
       </c>
       <c r="E239" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -5421,11 +5421,11 @@
         <v>10</v>
       </c>
       <c r="E273" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -6041,11 +6041,11 @@
         <v>10</v>
       </c>
       <c r="E307" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -6661,11 +6661,11 @@
         <v>10</v>
       </c>
       <c r="E341" t="n">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -7281,11 +7281,11 @@
         <v>10</v>
       </c>
       <c r="E375" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -7901,11 +7901,11 @@
         <v>10</v>
       </c>
       <c r="E409" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -8521,11 +8521,11 @@
         <v>10</v>
       </c>
       <c r="E443" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -9141,11 +9141,11 @@
         <v>10</v>
       </c>
       <c r="E477" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -9761,11 +9761,11 @@
         <v>10</v>
       </c>
       <c r="E511" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -10381,11 +10381,11 @@
         <v>10</v>
       </c>
       <c r="E545" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -11001,11 +11001,11 @@
         <v>10</v>
       </c>
       <c r="E579" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F579" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -11621,11 +11621,11 @@
         <v>10</v>
       </c>
       <c r="E613" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -12241,11 +12241,11 @@
         <v>10</v>
       </c>
       <c r="E647" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -12861,11 +12861,11 @@
         <v>10</v>
       </c>
       <c r="E681" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F681" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -13481,11 +13481,11 @@
         <v>10</v>
       </c>
       <c r="E715" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -14101,11 +14101,11 @@
         <v>10</v>
       </c>
       <c r="E749" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -14721,11 +14721,11 @@
         <v>10</v>
       </c>
       <c r="E783" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -15345,7 +15345,7 @@
       </c>
       <c r="F817" t="inlineStr">
         <is>
-          <t>2026-10-19 13:44</t>
+          <t>2026-10-20 11:33</t>
         </is>
       </c>
     </row>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>620</v>
+        <v>647</v>
       </c>
     </row>
     <row r="3">
@@ -15792,7 +15792,7 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>581</v>
+        <v>611</v>
       </c>
     </row>
     <row r="4">
@@ -15901,7 +15901,7 @@
         <v>0</v>
       </c>
       <c r="AI4" t="n">
-        <v>367</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5">
@@ -16010,7 +16010,7 @@
         <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6">
@@ -16119,7 +16119,7 @@
         <v>3555</v>
       </c>
       <c r="AI6" t="n">
-        <v>1938</v>
+        <v>2027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>